<commit_message>
wb = load_workbook(file_path, data_only=True)
</commit_message>
<xml_diff>
--- a/llm_result_ServiceCode2.xlsx
+++ b/llm_result_ServiceCode2.xlsx
@@ -1,39 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plumx\git_rep\ai_check_bot\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84051C3-DC57-479C-A89F-FDA7DA179D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="77">
   <si>
     <t>行番号</t>
   </si>
@@ -56,38 +37,226 @@
     <t>修正アドバイス</t>
   </si>
   <si>
+    <t>8888</t>
+  </si>
+  <si>
+    <t>1234</t>
+  </si>
+  <si>
     <t>1000000001</t>
   </si>
   <si>
+    <t>2000000001</t>
+  </si>
+  <si>
+    <t>0000000000</t>
+  </si>
+  <si>
+    <t>3000000001</t>
+  </si>
+  <si>
+    <t>3000000002</t>
+  </si>
+  <si>
+    <t>3000000003</t>
+  </si>
+  <si>
+    <t>3000000004</t>
+  </si>
+  <si>
+    <t>4000000001</t>
+  </si>
+  <si>
+    <t>4000000002</t>
+  </si>
+  <si>
+    <t>5000000001</t>
+  </si>
+  <si>
+    <t>5000000002</t>
+  </si>
+  <si>
+    <t>5000000003</t>
+  </si>
+  <si>
+    <t>6000000001</t>
+  </si>
+  <si>
+    <t>7000000001</t>
+  </si>
+  <si>
     <t>WBSマスタ登録可否フラグ</t>
   </si>
   <si>
+    <t>費用仕訳レベル</t>
+  </si>
+  <si>
+    <t>事業区分レベル</t>
+  </si>
+  <si>
+    <t>収益フラグ</t>
+  </si>
+  <si>
+    <t>費用フラグ</t>
+  </si>
+  <si>
+    <t>固定資産フラグ</t>
+  </si>
+  <si>
+    <t>区分経理フラグ</t>
+  </si>
+  <si>
+    <t>税金グループ</t>
+  </si>
+  <si>
+    <t>収益フラグ、費用フラグ</t>
+  </si>
+  <si>
     <t>Y</t>
   </si>
   <si>
+    <t>9999999999</t>
+  </si>
+  <si>
+    <t>1111111111</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>73A</t>
+  </si>
+  <si>
+    <t>73B</t>
+  </si>
+  <si>
+    <t>NULL, NULL</t>
+  </si>
+  <si>
     <t>チェック2：親値＝Yの場合、WBSマスタ登録可否フラグはNULLでなければならない。</t>
   </si>
   <si>
+    <t>チェック3：親値＝Nの場合、サービスコードと費用仕訳レベルは一致しなければならない。</t>
+  </si>
+  <si>
+    <t>チェック4－01：サービスコード＝0000000000の場合、費用仕訳レベルも0000000000でなければならない。</t>
+  </si>
+  <si>
+    <t>チェック4－02：サービスコード＝0000000000の場合、事業区分レベルはNULLでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック4－03：サービスコード＝0000000000の場合、収益フラグにYを設定することはできない。</t>
+  </si>
+  <si>
+    <t>チェック4－04：サービスコード＝0000000000の場合、費用フラグはYでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック4－05：サービスコード＝0000000000の場合、固定資産フラグにYを設定することはできない。</t>
+  </si>
+  <si>
+    <t>チェック4－06：サービスコード＝0000000000の場合、区分経理フラグにYを設定することはできない。</t>
+  </si>
+  <si>
+    <t>チェック4－07：サービスコード＝0000000000の場合、税金グループはNULLでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック4－08：サービスコード＝0000000000の場合、WBSマスタ登録可否フラグはYでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック5－01：固定資産フラグ=Yかつ会社コードが再編4社の場合、区分経理フラグはYでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック5－02：固定資産フラグ=Yかつ会社コードが再編4社の場合、サービスコードと事業区分レベルは一致しなければならない。</t>
+  </si>
+  <si>
+    <t>チェック5－03：固定資産フラグ=Yかつ会社コードが再編4社以外の場合、区分経理フラグにYを設定することはできない。</t>
+  </si>
+  <si>
+    <t>チェック5－04：固定資産フラグ=Yかつ会社コードが再編4社以外の場合、サービスコードは9988999999でなければならない。</t>
+  </si>
+  <si>
+    <t>チェック6－01：収益フラグ=NULLかつ費用フラグ=Yの場合、税金グループはNULLでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック6－02：収益フラグ=NULLかつ費用フラグ=Yの場合、WBSマスタ登録可否フラグはYでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック7－01：収益フラグ=Yの場合、税金グループは末尾がAでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック7－02：収益フラグ=Yの場合、WBSマスタ登録可否フラグはYでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック7－03：収益フラグがY以外の場合、税金グループはNULLでなければならない。</t>
+  </si>
+  <si>
+    <t>チェック8-01：会社コードが再編4社以外で、親値がN（子値）の場合、事業区分レベルは0000000000である必要があるため。</t>
+  </si>
+  <si>
+    <t>チェック9-01：親値がN（子値）の場合、収益フラグと費用フラグが共にNULL（未入力）は不可のため。※再編4社かつ区分経理フラグYの例外にも該当しません。</t>
+  </si>
+  <si>
     <t>WBSマスタ登録可否フラグをNULLに修正してください。</t>
+  </si>
+  <si>
+    <t>費用仕訳レベルをサービスコードと同じ値（2000000001）に修正してください。</t>
+  </si>
+  <si>
+    <t>費用仕訳レベルを0000000000に修正してください。</t>
+  </si>
+  <si>
+    <t>事業区分レベルをNULLに修正してください。</t>
+  </si>
+  <si>
+    <t>収益フラグをNULLに修正してください。</t>
+  </si>
+  <si>
+    <t>費用フラグをYに修正してください。</t>
+  </si>
+  <si>
+    <t>固定資産フラグをNULLに修正してください。</t>
+  </si>
+  <si>
+    <t>区分経理フラグをNULLに修正してください。</t>
+  </si>
+  <si>
+    <t>税金グループをNULLに修正してください。</t>
+  </si>
+  <si>
+    <t>WBSマスタ登録可否フラグをYに修正してください。</t>
+  </si>
+  <si>
+    <t>区分経理フラグをYに修正してください。</t>
+  </si>
+  <si>
+    <t>事業区分レベルをサービスコードと同じ3000000002に修正してください。</t>
+  </si>
+  <si>
+    <t>区分経理フラグをNULLまたはNに修正してください。</t>
+  </si>
+  <si>
+    <t>サービスコードを9988999999に修正してください。</t>
+  </si>
+  <si>
+    <t>税金グループを末尾Aの値に修正してください。</t>
+  </si>
+  <si>
+    <t>事業区分レベルを0000000000に修正してください。</t>
+  </si>
+  <si>
+    <t>収益フラグまたは費用フラグのいずれかにYを設定してください。</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="ＭＳ Ｐゴシック"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -115,25 +284,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -171,7 +332,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -205,7 +366,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -240,10 +400,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -416,16 +575,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -448,7 +602,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>8</v>
       </c>
@@ -456,23 +610,482 @@
         <v>1234</v>
       </c>
       <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>1234</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>1234</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>1234</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>1234</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>1234</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>1234</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>1234</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>1234</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>17</v>
+      </c>
+      <c r="B11">
+        <v>1234</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12">
+        <v>18</v>
+      </c>
+      <c r="B12">
+        <v>1001</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13">
+        <v>19</v>
+      </c>
+      <c r="B13">
+        <v>1002</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14">
+        <v>20</v>
+      </c>
+      <c r="B14">
+        <v>8888</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15">
+        <v>21</v>
+      </c>
+      <c r="B15">
+        <v>8888</v>
+      </c>
+      <c r="C15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16">
+        <v>22</v>
+      </c>
+      <c r="B16">
+        <v>1234</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17">
+        <v>23</v>
+      </c>
+      <c r="B17">
+        <v>1234</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" t="s">
+        <v>54</v>
+      </c>
+      <c r="G17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18">
+        <v>24</v>
+      </c>
+      <c r="B18">
+        <v>1234</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19">
+        <v>25</v>
+      </c>
+      <c r="B19">
+        <v>1234</v>
+      </c>
+      <c r="C19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20">
+        <v>26</v>
+      </c>
+      <c r="B20">
+        <v>1234</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" t="s">
+        <v>36</v>
+      </c>
+      <c r="F20" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" t="s">
+        <v>58</v>
+      </c>
+      <c r="G21" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>28</v>
+      </c>
+      <c r="B22" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
+      <c r="C22" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22" t="s">
+        <v>59</v>
+      </c>
+      <c r="G22" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>